<commit_message>
Updated FINANCIAL FUNCTIONS QUESTIONS.xlsx
</commit_message>
<xml_diff>
--- a/FINANCIAL FUNCTIONS QUESTIONS.xlsx
+++ b/FINANCIAL FUNCTIONS QUESTIONS.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27628"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Besant\Besant Excel\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Besant\Excel\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7C2B5662-84B4-4E3E-A2F9-63A4A0A8FE72}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{31E67DC5-167A-47BA-9D49-9438F1D52614}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-98" yWindow="-98" windowWidth="24196" windowHeight="14476" xr2:uid="{29C95F6E-244C-4ECB-89DA-68F6A5B818FF}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11020" xr2:uid="{29C95F6E-244C-4ECB-89DA-68F6A5B818FF}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="36" uniqueCount="14">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="42" uniqueCount="19">
   <si>
     <t>Prinicipal Amount</t>
   </si>
@@ -77,6 +77,21 @@
   </si>
   <si>
     <t>FINACIAL FUNCTIONS</t>
+  </si>
+  <si>
+    <t>FV(C10,D10,B10)</t>
+  </si>
+  <si>
+    <t>PMT(C13/12,D13*12,B12)</t>
+  </si>
+  <si>
+    <t>PPMT(C16/12,1,D16*12,B16)</t>
+  </si>
+  <si>
+    <t>IPMT(C19/12,1,D19*12,B19)</t>
+  </si>
+  <si>
+    <t>FV(C22,D22,,B22)</t>
   </si>
 </sst>
 </file>
@@ -84,11 +99,11 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="5">
-    <numFmt numFmtId="8" formatCode="&quot;₹&quot;\ #,##0.00;[Red]&quot;₹&quot;\ \-#,##0.00"/>
-    <numFmt numFmtId="164" formatCode="[$₹-44B]#,##0.00;[Red][$₹-44B]\-#,##0.00"/>
-    <numFmt numFmtId="165" formatCode="[$₹-44B]#,##0.00"/>
-    <numFmt numFmtId="166" formatCode="&quot;£&quot;#,##0.00;[Red]\-&quot;£&quot;#,##0.00"/>
-    <numFmt numFmtId="167" formatCode="0.0%"/>
+    <numFmt numFmtId="164" formatCode="&quot;₹&quot;\ #,##0.00;[Red]&quot;₹&quot;\ \-#,##0.00"/>
+    <numFmt numFmtId="165" formatCode="[$₹-44B]#,##0.00;[Red][$₹-44B]\-#,##0.00"/>
+    <numFmt numFmtId="166" formatCode="[$₹-44B]#,##0.00"/>
+    <numFmt numFmtId="167" formatCode="&quot;£&quot;#,##0.00;[Red]\-&quot;£&quot;#,##0.00"/>
+    <numFmt numFmtId="168" formatCode="0.0%"/>
   </numFmts>
   <fonts count="3" x14ac:knownFonts="1">
     <font>
@@ -259,17 +274,17 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1"/>
     <xf numFmtId="10" fontId="0" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1"/>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyBorder="1"/>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="9" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="8" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="10" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyBorder="1"/>
-    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="167" fontId="0" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyBorder="1"/>
-    <xf numFmtId="167" fontId="0" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="167" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="168" fontId="0" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="168" fontId="0" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyBorder="1"/>
     <xf numFmtId="1" fontId="0" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -360,9 +375,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 2013 - 2022 Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
   <a:themeElements>
-    <a:clrScheme name="Office 2013 - 2022">
+    <a:clrScheme name="Office">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -400,7 +415,7 @@
         <a:srgbClr val="954F72"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office 2013 - 2022">
+    <a:fontScheme name="Office">
       <a:majorFont>
         <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
@@ -506,7 +521,7 @@
         <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office 2013 - 2022">
+    <a:fmtScheme name="Office">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -648,7 +663,7 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office 2013 - 2022 Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
@@ -657,17 +672,17 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{19061382-15BA-4790-91D1-B6A3F04B2D57}">
   <dimension ref="A4:AD34"/>
-  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="2" max="2" width="15.53125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="12.796875" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="12.19921875" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="25.06640625" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="9.73046875" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="11.59765625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="15.54296875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="12.81640625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="12.1796875" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="25.08984375" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="9.7265625" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="11.6328125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="4" spans="1:30" x14ac:dyDescent="0.45">
+    <row r="4" spans="1:30" x14ac:dyDescent="0.35">
       <c r="A4" s="21" t="s">
         <v>13</v>
       </c>
@@ -677,7 +692,7 @@
       <c r="E4" s="21"/>
       <c r="F4" s="21"/>
     </row>
-    <row r="5" spans="1:30" x14ac:dyDescent="0.45">
+    <row r="5" spans="1:30" x14ac:dyDescent="0.35">
       <c r="A5" s="21"/>
       <c r="B5" s="21"/>
       <c r="C5" s="21"/>
@@ -685,8 +700,8 @@
       <c r="E5" s="21"/>
       <c r="F5" s="21"/>
     </row>
-    <row r="8" spans="1:30" ht="14.65" thickBot="1" x14ac:dyDescent="0.5"/>
-    <row r="9" spans="1:30" x14ac:dyDescent="0.45">
+    <row r="8" spans="1:30" ht="15" thickBot="1" x14ac:dyDescent="0.4"/>
+    <row r="9" spans="1:30" x14ac:dyDescent="0.35">
       <c r="B9" s="1" t="s">
         <v>0</v>
       </c>
@@ -696,9 +711,11 @@
       <c r="D9" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="E9" s="3"/>
-    </row>
-    <row r="10" spans="1:30" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
+      <c r="E9" s="3" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="10" spans="1:30" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="B10" s="4">
         <v>-65000</v>
       </c>
@@ -708,10 +725,16 @@
       <c r="D10" s="6">
         <v>5</v>
       </c>
-      <c r="E10" s="7"/>
-      <c r="F10" s="8" t="e">
+      <c r="E10" s="7">
+        <f>FV(C10,D10,,B10)</f>
+        <v>100010.55706850003</v>
+      </c>
+      <c r="F10" s="8" t="str">
         <f ca="1">_xlfn.FORMULATEXT(E10)</f>
-        <v>#N/A</v>
+        <v>=FV(C10,D10,,B10)</v>
+      </c>
+      <c r="G10" t="s">
+        <v>14</v>
       </c>
       <c r="H10" s="9"/>
       <c r="J10" s="10"/>
@@ -742,12 +765,12 @@
         <v>80</v>
       </c>
     </row>
-    <row r="11" spans="1:30" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
+    <row r="11" spans="1:30" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="C11" s="12"/>
       <c r="E11" s="13"/>
       <c r="F11" s="8"/>
     </row>
-    <row r="12" spans="1:30" x14ac:dyDescent="0.45">
+    <row r="12" spans="1:30" x14ac:dyDescent="0.35">
       <c r="A12" s="22">
         <v>46</v>
       </c>
@@ -764,7 +787,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="13" spans="1:30" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
+    <row r="13" spans="1:30" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A13" s="23"/>
       <c r="B13" s="6">
         <v>65000</v>
@@ -775,17 +798,23 @@
       <c r="D13" s="6">
         <v>3</v>
       </c>
-      <c r="E13" s="7"/>
-      <c r="F13" t="e">
+      <c r="E13" s="7">
+        <f>PMT(C13/12,D13*12,B13)</f>
+        <v>-2051.8899325312309</v>
+      </c>
+      <c r="F13" t="str">
         <f ca="1">_xlfn.FORMULATEXT(E13)</f>
-        <v>#N/A</v>
-      </c>
-    </row>
-    <row r="14" spans="1:30" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
+        <v>=PMT(C13/12,D13*12,B13)</v>
+      </c>
+      <c r="G13" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="14" spans="1:30" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="C14" s="12"/>
       <c r="E14" s="13"/>
     </row>
-    <row r="15" spans="1:30" x14ac:dyDescent="0.45">
+    <row r="15" spans="1:30" x14ac:dyDescent="0.35">
       <c r="A15" s="19">
         <v>47</v>
       </c>
@@ -802,7 +831,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="16" spans="1:30" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
+    <row r="16" spans="1:30" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A16" s="20"/>
       <c r="B16" s="6">
         <v>65000</v>
@@ -813,17 +842,23 @@
       <c r="D16" s="6">
         <v>3</v>
       </c>
-      <c r="E16" s="7"/>
-      <c r="F16" t="e">
+      <c r="E16" s="7">
+        <f>PPMT(C16/12,1,D16*12,B16)</f>
+        <v>-1591.4732658645644</v>
+      </c>
+      <c r="F16" t="str">
         <f ca="1">_xlfn.FORMULATEXT(E16)</f>
-        <v>#N/A</v>
-      </c>
-    </row>
-    <row r="17" spans="1:7" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
+        <v>=PPMT(C16/12,1,D16*12,B16)</v>
+      </c>
+      <c r="G16" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="17" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="C17" s="12"/>
       <c r="E17" s="13"/>
     </row>
-    <row r="18" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="18" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A18" s="19">
         <v>48</v>
       </c>
@@ -840,7 +875,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="19" spans="1:7" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
+    <row r="19" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A19" s="20"/>
       <c r="B19" s="6">
         <v>65000</v>
@@ -851,17 +886,23 @@
       <c r="D19" s="6">
         <v>3</v>
       </c>
-      <c r="E19" s="7"/>
-      <c r="F19" t="e">
+      <c r="E19" s="7">
+        <f>IPMT(C19/12,1,D19*12,B19)</f>
+        <v>-460.41666666666674</v>
+      </c>
+      <c r="F19" t="str">
         <f ca="1">_xlfn.FORMULATEXT(E19)</f>
-        <v>#N/A</v>
-      </c>
-    </row>
-    <row r="20" spans="1:7" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
+        <v>=IPMT(C19/12,1,D19*12,B19)</v>
+      </c>
+      <c r="G19" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="20" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="C20" s="12"/>
       <c r="E20" s="13"/>
     </row>
-    <row r="21" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="21" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A21" s="19">
         <v>49</v>
       </c>
@@ -878,7 +919,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="22" spans="1:7" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
+    <row r="22" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A22" s="20"/>
       <c r="B22" s="6">
         <v>-25000</v>
@@ -889,17 +930,23 @@
       <c r="D22" s="6">
         <v>5</v>
       </c>
-      <c r="E22" s="7"/>
-      <c r="F22" t="e">
+      <c r="E22" s="7">
+        <f>FV(C22,D22,,B22)</f>
+        <v>37160.327581525875</v>
+      </c>
+      <c r="F22" t="str">
         <f ca="1">_xlfn.FORMULATEXT(E22)</f>
-        <v>#N/A</v>
-      </c>
-    </row>
-    <row r="23" spans="1:7" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
+        <v>=FV(C22,D22,,B22)</v>
+      </c>
+      <c r="G22" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="23" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="C23" s="12"/>
       <c r="E23" s="13"/>
     </row>
-    <row r="24" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="24" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A24" s="19">
         <v>50</v>
       </c>
@@ -916,7 +963,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="25" spans="1:7" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
+    <row r="25" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A25" s="20"/>
       <c r="B25" s="6">
         <v>-1200</v>
@@ -927,17 +974,20 @@
       <c r="D25" s="6">
         <v>5</v>
       </c>
-      <c r="E25" s="7"/>
-      <c r="F25" t="e">
+      <c r="E25" s="7">
+        <f>FV(C25,D25,,B25)</f>
+        <v>1722.7551914062499</v>
+      </c>
+      <c r="F25" t="str">
         <f ca="1">_xlfn.FORMULATEXT(E25)</f>
-        <v>#N/A</v>
-      </c>
-    </row>
-    <row r="26" spans="1:7" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
+        <v>=FV(C25,D25,,B25)</v>
+      </c>
+    </row>
+    <row r="26" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="C26" s="12"/>
       <c r="E26" s="15"/>
     </row>
-    <row r="27" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="27" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A27" s="19">
         <v>51</v>
       </c>
@@ -954,7 +1004,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="28" spans="1:7" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
+    <row r="28" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A28" s="20"/>
       <c r="B28" s="6">
         <v>-1476</v>
@@ -971,10 +1021,10 @@
         <v>#N/A</v>
       </c>
     </row>
-    <row r="29" spans="1:7" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
+    <row r="29" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="E29" s="9"/>
     </row>
-    <row r="30" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="30" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A30" s="19">
         <v>52</v>
       </c>
@@ -991,7 +1041,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="31" spans="1:7" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
+    <row r="31" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A31" s="20"/>
       <c r="B31" s="6">
         <v>10</v>
@@ -1009,11 +1059,11 @@
       </c>
       <c r="G31" s="10"/>
     </row>
-    <row r="32" spans="1:7" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
+    <row r="32" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="D32" s="12"/>
       <c r="E32" s="13"/>
     </row>
-    <row r="33" spans="1:6" x14ac:dyDescent="0.45">
+    <row r="33" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A33" s="19">
         <v>53</v>
       </c>
@@ -1030,7 +1080,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="34" spans="1:6" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
+    <row r="34" spans="1:6" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A34" s="20"/>
       <c r="B34" s="6">
         <v>-1520</v>
@@ -1067,7 +1117,7 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9CBDE502-262C-4CEF-88CE-D15095966CCB}">
   <dimension ref="A1"/>
-  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <sheetData/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>